<commit_message>
feat(viceri-study): publish specification and test suite v1.5
</commit_message>
<xml_diff>
--- a/output/xlsx/AdministradorRealizaPickingDeEcommerce--GT-.xlsx
+++ b/output/xlsx/AdministradorRealizaPickingDeEcommerce--GT-.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="68">
   <si>
     <t xml:space="preserve">System: </t>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Use Case: </t>
   </si>
   <si>
-    <t>Administrador Realiza Picking De Ecommerce</t>
+    <t>Administrador Registra Ocorrencia Em Nota De Coleta</t>
   </si>
   <si>
     <t xml:space="preserve">Version: </t>
@@ -38,7 +38,7 @@
     <t>Reduced (Greedy Heuristic - Transition Coverage)</t>
   </si>
   <si>
-    <t>Size: 8 test case(s)</t>
+    <t>Size: 11 test case(s)</t>
   </si>
   <si>
     <t xml:space="preserve">Creation Date: </t>
@@ -92,106 +92,130 @@
     <t>Actual Result</t>
   </si>
   <si>
-    <t>Administrador: clica na opcao 'Picking' no menu da tela principal</t>
+    <t>Administrador: clica na opcao 'Central de Operacoes' no menu da tela principal</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>SYSTEM exibe lista de Ecommerces registrados no sistema</t>
-  </si>
-  <si>
-    <t>Administrador: clica em algum dos Ecommerces listados</t>
-  </si>
-  <si>
-    <t>SYSTEM abre uma tela com o Picking diario para aquele Ecommerce selecionado</t>
-  </si>
-  <si>
-    <t>Administrador: clica no botao 'Iniciar Picking'</t>
-  </si>
-  <si>
-    <t>SYSTEM exibe os dados do Picking</t>
-  </si>
-  <si>
-    <t>Administrador: clica no botao de 'Finalizar Picking'</t>
-  </si>
-  <si>
-    <t>SYSTEM notifica que Picking foi finalizado com sucesso e exibe Dashboard de sistema</t>
+    <t>SYSTEM exibe Dashboard do sistema</t>
+  </si>
+  <si>
+    <t>Administrador: clica em contador 'Geradas' na secao de 'Coletas'</t>
+  </si>
+  <si>
+    <t>SYSTEM abre uma tela com as listas das 'Coletas'</t>
+  </si>
+  <si>
+    <t>Administrador: seleciona alguma Coleta da lista</t>
+  </si>
+  <si>
+    <t>SYSTEM exibe os dados da Coleta</t>
+  </si>
+  <si>
+    <t>Administrador: clica no botao de 'Registrar Ocorrencia' associado a qualquer item da nota</t>
+  </si>
+  <si>
+    <t>SYSTEM abre modal para digitacao da ocorrencia</t>
+  </si>
+  <si>
+    <t>Administrador: digita ocorrencia e clica em 'Confirmar'</t>
+  </si>
+  <si>
+    <t>SYSTEM notifica que Ocorrencia foi registrada com sucesso</t>
   </si>
   <si>
     <t xml:space="preserve">Postcondition: </t>
   </si>
   <si>
-    <t>O Picking diario foi realizado para o Ecommerce</t>
+    <t>A ocorrencia esta registrada e nota esta com status de ocorrencia registrada</t>
   </si>
   <si>
     <t>TC2</t>
   </si>
   <si>
-    <t>Alternative Flow 1: Navega pelas paginas da lista</t>
+    <t>Alternative Flow 1: Seleciona contador de 'Aguardando Picking'</t>
+  </si>
+  <si>
+    <t>Administrador: clica em algum contador de 'Aguardando Picking' na secao de 'Coletas'</t>
+  </si>
+  <si>
+    <t>TC3</t>
+  </si>
+  <si>
+    <t>Alternative Flow 2: Seleciona contador de 'Aceitas'</t>
+  </si>
+  <si>
+    <t>Administrador: clica em algum contador de 'Aceitas' na secao de 'Coletas'</t>
+  </si>
+  <si>
+    <t>TC4</t>
+  </si>
+  <si>
+    <t>Alternative Flow 3: Seleciona contador de 'Recusadas'</t>
+  </si>
+  <si>
+    <t>Administrador: clica em algum contador de 'Recusadas' na secao de 'Coletas'</t>
+  </si>
+  <si>
+    <t>TC5</t>
+  </si>
+  <si>
+    <t>Alternative Flow 4: Seleciona contador de 'A Caminho'</t>
+  </si>
+  <si>
+    <t>Administrador: clica em algum contador de 'A Caminho' na secao de 'Coletas'</t>
+  </si>
+  <si>
+    <t>TC6</t>
+  </si>
+  <si>
+    <t>Alternative Flow 5: Navega pelas paginas da lista</t>
   </si>
   <si>
     <t>Administrador: seleciona outra pagina</t>
   </si>
   <si>
-    <t>TC3</t>
-  </si>
-  <si>
-    <t>Alternative Flow 2: Clica no botao 'Voltar'</t>
+    <t>TC7</t>
+  </si>
+  <si>
+    <t>Alternative Flow 6: Clica no botao 'Voltar'</t>
   </si>
   <si>
     <t>Administrador: clica no botao 'Voltar'</t>
   </si>
   <si>
-    <t>TC4</t>
-  </si>
-  <si>
-    <t>Alternative Flow 3: Ordena os Ecommerces</t>
-  </si>
-  <si>
-    <t>Administrador: ordena os Ecommerces por alguma coluna</t>
-  </si>
-  <si>
-    <t>TC5</t>
-  </si>
-  <si>
-    <t>Alternative Flow 4: Filtra coletas da lista</t>
+    <t>TC8</t>
+  </si>
+  <si>
+    <t>Alternative Flow 7: Ordena Coletas</t>
+  </si>
+  <si>
+    <t>Administrador: ordena as Coletas por alguma coluna</t>
+  </si>
+  <si>
+    <t>TC9</t>
+  </si>
+  <si>
+    <t>Alternative Flow 8: Cancela registro de ocorrencia</t>
+  </si>
+  <si>
+    <t>Administrador: clica em botao 'Cancelar'</t>
+  </si>
+  <si>
+    <t>TC10</t>
+  </si>
+  <si>
+    <t>Alternative Flow 9: Volta para lista de Coletas</t>
+  </si>
+  <si>
+    <t>TC11</t>
+  </si>
+  <si>
+    <t>Alternative Flow 10: Filtra coletas da lista</t>
   </si>
   <si>
     <t>Administrador: filtra as coletas por algum campo</t>
-  </si>
-  <si>
-    <t>TC6</t>
-  </si>
-  <si>
-    <t>Alternative Flow 5: Cancela realizacao de Picking</t>
-  </si>
-  <si>
-    <t>Administrador: clica em botao 'Cancelar'</t>
-  </si>
-  <si>
-    <t>TC8</t>
-  </si>
-  <si>
-    <t>Alternative Flow 7: Clica no botao 'Proximo Picking'</t>
-  </si>
-  <si>
-    <t>Administrador: clica no botao 'Proximo Picking'</t>
-  </si>
-  <si>
-    <t>TC9</t>
-  </si>
-  <si>
-    <t>Alternative Flow 8: realiza picking depois de consultar veiculos</t>
-  </si>
-  <si>
-    <t>Administrador: clica em botao 'Consultar Veiculos'</t>
-  </si>
-  <si>
-    <t>SYSTEM exibe lista de veiculos para picking</t>
-  </si>
-  <si>
-    <t>Administrador: clica em botao 'Iniciar Picking'</t>
   </si>
 </sst>
 </file>
@@ -283,13 +307,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F144"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="52.5546875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="72.875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="21.8984375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="69.05078125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="48.1796875" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="30.5234375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="17.578125" customWidth="true" bestFit="true"/>
   </cols>
@@ -467,92 +491,92 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="s" s="1">
+      <c r="A14" t="n" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="B14" t="s" s="3">
         <v>35</v>
       </c>
-      <c r="B14" t="s" s="0">
+      <c r="C14" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D14" t="s" s="3">
         <v>36</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B17" t="s" s="0">
+      <c r="E14" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F14" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="1">
         <v>37</v>
       </c>
-      <c r="C17" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E17" t="s" s="1">
-        <v>14</v>
+      <c r="B15" t="s" s="0">
+        <v>38</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="1">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="C18" t="s" s="1">
+        <v>13</v>
       </c>
       <c r="E18" t="s" s="1">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E19" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="B19" t="s" s="0">
+      <c r="B20" t="s" s="0">
         <v>19</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="s" s="2">
+    <row r="21">
+      <c r="A21" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B20" t="s" s="2">
+      <c r="B21" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="C20" t="s" s="2">
+      <c r="C21" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D20" t="s" s="2">
+      <c r="D21" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="E20" t="s" s="2">
+      <c r="E21" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="F20" t="s" s="2">
+      <c r="F21" t="s" s="2">
         <v>25</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B21" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C21" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D21" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E21" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F21" t="s" s="3">
-        <v>27</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n" s="4">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B22" t="s" s="3">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="C22" t="s" s="3">
         <v>27</v>
@@ -569,10 +593,10 @@
     </row>
     <row r="23">
       <c r="A23" t="n" s="4">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="B23" t="s" s="3">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="C23" t="s" s="3">
         <v>27</v>
@@ -589,7 +613,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n" s="4">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="B24" t="s" s="3">
         <v>31</v>
@@ -609,7 +633,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n" s="4">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="B25" t="s" s="3">
         <v>33</v>
@@ -628,92 +652,92 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="s" s="1">
+      <c r="A26" t="n" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="B26" t="s" s="3">
         <v>35</v>
       </c>
-      <c r="B26" t="s" s="0">
+      <c r="C26" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D26" t="s" s="3">
         <v>36</v>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B29" t="s" s="0">
-        <v>40</v>
-      </c>
-      <c r="C29" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E29" t="s" s="1">
-        <v>14</v>
+      <c r="E26" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F26" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>38</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="1">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="C30" t="s" s="1">
+        <v>13</v>
       </c>
       <c r="E30" t="s" s="1">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="E31" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="B31" t="s" s="0">
+      <c r="B32" t="s" s="0">
         <v>19</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="s" s="2">
+    <row r="33">
+      <c r="A33" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B32" t="s" s="2">
+      <c r="B33" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="C32" t="s" s="2">
+      <c r="C33" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D32" t="s" s="2">
+      <c r="D33" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="E32" t="s" s="2">
+      <c r="E33" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="F32" t="s" s="2">
+      <c r="F33" t="s" s="2">
         <v>25</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B33" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C33" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D33" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E33" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F33" t="s" s="3">
-        <v>27</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n" s="4">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B34" t="s" s="3">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="C34" t="s" s="3">
         <v>27</v>
@@ -730,10 +754,10 @@
     </row>
     <row r="35">
       <c r="A35" t="n" s="4">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="B35" t="s" s="3">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="C35" t="s" s="3">
         <v>27</v>
@@ -750,7 +774,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n" s="4">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="B36" t="s" s="3">
         <v>31</v>
@@ -770,7 +794,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n" s="4">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="B37" t="s" s="3">
         <v>33</v>
@@ -789,92 +813,92 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="s" s="1">
+      <c r="A38" t="n" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="B38" t="s" s="3">
         <v>35</v>
       </c>
-      <c r="B38" t="s" s="0">
+      <c r="C38" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D38" t="s" s="3">
         <v>36</v>
       </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B41" t="s" s="0">
-        <v>43</v>
-      </c>
-      <c r="C41" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E41" t="s" s="1">
-        <v>14</v>
+      <c r="E38" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F38" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>38</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="1">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="C42" t="s" s="1">
+        <v>13</v>
       </c>
       <c r="E42" t="s" s="1">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B43" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="E43" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="B43" t="s" s="0">
+      <c r="B44" t="s" s="0">
         <v>19</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="s" s="2">
+    <row r="45">
+      <c r="A45" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B44" t="s" s="2">
+      <c r="B45" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="C44" t="s" s="2">
+      <c r="C45" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D44" t="s" s="2">
+      <c r="D45" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="E44" t="s" s="2">
+      <c r="E45" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="F44" t="s" s="2">
+      <c r="F45" t="s" s="2">
         <v>25</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B45" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C45" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D45" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E45" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F45" t="s" s="3">
-        <v>27</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n" s="4">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B46" t="s" s="3">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="C46" t="s" s="3">
         <v>27</v>
@@ -891,10 +915,10 @@
     </row>
     <row r="47">
       <c r="A47" t="n" s="4">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="B47" t="s" s="3">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="C47" t="s" s="3">
         <v>27</v>
@@ -911,7 +935,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n" s="4">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="B48" t="s" s="3">
         <v>31</v>
@@ -931,7 +955,7 @@
     </row>
     <row r="49">
       <c r="A49" t="n" s="4">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="B49" t="s" s="3">
         <v>33</v>
@@ -950,92 +974,92 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="s" s="1">
+      <c r="A50" t="n" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="B50" t="s" s="3">
         <v>35</v>
       </c>
-      <c r="B50" t="s" s="0">
+      <c r="C50" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D50" t="s" s="3">
         <v>36</v>
       </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B53" t="s" s="0">
-        <v>46</v>
-      </c>
-      <c r="C53" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E53" t="s" s="1">
-        <v>14</v>
+      <c r="E50" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F50" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B51" t="s" s="0">
+        <v>38</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="1">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
+      </c>
+      <c r="C54" t="s" s="1">
+        <v>13</v>
       </c>
       <c r="E54" t="s" s="1">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B55" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="E55" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="B55" t="s" s="0">
+      <c r="B56" t="s" s="0">
         <v>19</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="s" s="2">
+    <row r="57">
+      <c r="A57" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B56" t="s" s="2">
+      <c r="B57" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="C56" t="s" s="2">
+      <c r="C57" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D56" t="s" s="2">
+      <c r="D57" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="E56" t="s" s="2">
+      <c r="E57" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="F56" t="s" s="2">
+      <c r="F57" t="s" s="2">
         <v>25</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B57" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C57" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D57" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E57" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F57" t="s" s="3">
-        <v>27</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n" s="4">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B58" t="s" s="3">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="C58" t="s" s="3">
         <v>27</v>
@@ -1052,10 +1076,10 @@
     </row>
     <row r="59">
       <c r="A59" t="n" s="4">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="B59" t="s" s="3">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="C59" t="s" s="3">
         <v>27</v>
@@ -1072,7 +1096,7 @@
     </row>
     <row r="60">
       <c r="A60" t="n" s="4">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="B60" t="s" s="3">
         <v>31</v>
@@ -1092,7 +1116,7 @@
     </row>
     <row r="61">
       <c r="A61" t="n" s="4">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="B61" t="s" s="3">
         <v>33</v>
@@ -1111,98 +1135,98 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="s" s="1">
+      <c r="A62" t="n" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="B62" t="s" s="3">
         <v>35</v>
       </c>
-      <c r="B62" t="s" s="0">
+      <c r="C62" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D62" t="s" s="3">
         <v>36</v>
       </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B65" t="s" s="0">
-        <v>49</v>
-      </c>
-      <c r="C65" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E65" t="s" s="1">
-        <v>14</v>
+      <c r="E62" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F62" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B63" t="s" s="0">
+        <v>38</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s" s="1">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B66" t="s" s="0">
-        <v>50</v>
+        <v>51</v>
+      </c>
+      <c r="C66" t="s" s="1">
+        <v>13</v>
       </c>
       <c r="E66" t="s" s="1">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B67" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E67" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="B67" t="s" s="0">
+      <c r="B68" t="s" s="0">
         <v>19</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="s" s="2">
+    <row r="69">
+      <c r="A69" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B68" t="s" s="2">
+      <c r="B69" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="C68" t="s" s="2">
+      <c r="C69" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D68" t="s" s="2">
+      <c r="D69" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="E68" t="s" s="2">
+      <c r="E69" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="F68" t="s" s="2">
+      <c r="F69" t="s" s="2">
         <v>25</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B69" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C69" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D69" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E69" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F69" t="s" s="3">
-        <v>27</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n" s="4">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B70" t="s" s="3">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C70" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D70" t="s" s="3">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E70" t="s" s="3">
         <v>27</v>
@@ -1213,16 +1237,16 @@
     </row>
     <row r="71">
       <c r="A71" t="n" s="4">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="B71" t="s" s="3">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="C71" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D71" t="s" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E71" t="s" s="3">
         <v>27</v>
@@ -1233,10 +1257,10 @@
     </row>
     <row r="72">
       <c r="A72" t="n" s="4">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="B72" t="s" s="3">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="C72" t="s" s="3">
         <v>27</v>
@@ -1253,7 +1277,7 @@
     </row>
     <row r="73">
       <c r="A73" t="n" s="4">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="B73" t="s" s="3">
         <v>31</v>
@@ -1273,7 +1297,7 @@
     </row>
     <row r="74">
       <c r="A74" t="n" s="4">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="B74" t="s" s="3">
         <v>33</v>
@@ -1292,98 +1316,98 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="s" s="1">
+      <c r="A75" t="n" s="4">
+        <v>6.0</v>
+      </c>
+      <c r="B75" t="s" s="3">
         <v>35</v>
       </c>
-      <c r="B75" t="s" s="0">
+      <c r="C75" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D75" t="s" s="3">
         <v>36</v>
       </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B78" t="s" s="0">
-        <v>52</v>
-      </c>
-      <c r="C78" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E78" t="s" s="1">
-        <v>14</v>
+      <c r="E75" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F75" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B76" t="s" s="0">
+        <v>38</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s" s="1">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B79" t="s" s="0">
-        <v>53</v>
+        <v>54</v>
+      </c>
+      <c r="C79" t="s" s="1">
+        <v>13</v>
       </c>
       <c r="E79" t="s" s="1">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B80" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="E80" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="B80" t="s" s="0">
+      <c r="B81" t="s" s="0">
         <v>19</v>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" t="s" s="2">
+    <row r="82">
+      <c r="A82" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B81" t="s" s="2">
+      <c r="B82" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="C81" t="s" s="2">
+      <c r="C82" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D81" t="s" s="2">
+      <c r="D82" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="E81" t="s" s="2">
+      <c r="E82" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="F81" t="s" s="2">
+      <c r="F82" t="s" s="2">
         <v>25</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B82" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C82" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D82" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E82" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F82" t="s" s="3">
-        <v>27</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n" s="4">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B83" t="s" s="3">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C83" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D83" t="s" s="3">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E83" t="s" s="3">
         <v>27</v>
@@ -1394,16 +1418,16 @@
     </row>
     <row r="84">
       <c r="A84" t="n" s="4">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="B84" t="s" s="3">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C84" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D84" t="s" s="3">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E84" t="s" s="3">
         <v>27</v>
@@ -1414,16 +1438,16 @@
     </row>
     <row r="85">
       <c r="A85" t="n" s="4">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="B85" t="s" s="3">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C85" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D85" t="s" s="3">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E85" t="s" s="3">
         <v>27</v>
@@ -1434,157 +1458,157 @@
     </row>
     <row r="86">
       <c r="A86" t="n" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="B86" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="C86" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D86" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E86" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F86" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n" s="4">
         <v>5.0</v>
       </c>
-      <c r="B86" t="s" s="3">
+      <c r="B87" t="s" s="3">
+        <v>31</v>
+      </c>
+      <c r="C87" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D87" t="s" s="3">
+        <v>32</v>
+      </c>
+      <c r="E87" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F87" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n" s="4">
+        <v>6.0</v>
+      </c>
+      <c r="B88" t="s" s="3">
         <v>33</v>
       </c>
-      <c r="C86" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D86" t="s" s="3">
+      <c r="C88" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D88" t="s" s="3">
         <v>34</v>
       </c>
-      <c r="E86" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F86" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="s" s="1">
+      <c r="E88" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F88" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n" s="4">
+        <v>7.0</v>
+      </c>
+      <c r="B89" t="s" s="3">
         <v>35</v>
       </c>
-      <c r="B87" t="s" s="0">
+      <c r="C89" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D89" t="s" s="3">
         <v>36</v>
+      </c>
+      <c r="E89" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F89" t="s" s="3">
+        <v>27</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B90" t="s" s="0">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="s" s="1">
         <v>11</v>
       </c>
-      <c r="B90" t="s" s="0">
-        <v>55</v>
-      </c>
-      <c r="C90" t="s" s="1">
+      <c r="B93" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="C93" t="s" s="1">
         <v>13</v>
       </c>
-      <c r="E90" t="s" s="1">
+      <c r="E93" t="s" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" t="s" s="1">
+    <row r="94">
+      <c r="A94" t="s" s="1">
         <v>15</v>
       </c>
-      <c r="B91" t="s" s="0">
-        <v>56</v>
-      </c>
-      <c r="E91" t="s" s="1">
+      <c r="B94" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="E94" t="s" s="1">
         <v>17</v>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" t="s" s="1">
+    <row r="95">
+      <c r="A95" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="B92" t="s" s="0">
+      <c r="B95" t="s" s="0">
         <v>19</v>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" t="s" s="2">
+    <row r="96">
+      <c r="A96" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B93" t="s" s="2">
+      <c r="B96" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="C93" t="s" s="2">
+      <c r="C96" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D93" t="s" s="2">
+      <c r="D96" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="E93" t="s" s="2">
+      <c r="E96" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="F93" t="s" s="2">
+      <c r="F96" t="s" s="2">
         <v>25</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B94" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C94" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D94" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E94" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F94" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="n" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="B95" t="s" s="3">
-        <v>29</v>
-      </c>
-      <c r="C95" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D95" t="s" s="3">
-        <v>30</v>
-      </c>
-      <c r="E95" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F95" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="n" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="B96" t="s" s="3">
-        <v>57</v>
-      </c>
-      <c r="C96" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D96" t="s" s="3">
-        <v>58</v>
-      </c>
-      <c r="E96" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F96" t="s" s="3">
-        <v>27</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n" s="4">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="B97" t="s" s="3">
-        <v>59</v>
+        <v>26</v>
       </c>
       <c r="C97" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D97" t="s" s="3">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E97" t="s" s="3">
         <v>27</v>
@@ -1595,30 +1619,693 @@
     </row>
     <row r="98">
       <c r="A98" t="n" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="B98" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="C98" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D98" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E98" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F98" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="B99" t="s" s="3">
+        <v>59</v>
+      </c>
+      <c r="C99" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D99" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E99" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F99" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="B100" t="s" s="3">
+        <v>31</v>
+      </c>
+      <c r="C100" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D100" t="s" s="3">
+        <v>32</v>
+      </c>
+      <c r="E100" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F100" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n" s="4">
         <v>5.0</v>
       </c>
-      <c r="B98" t="s" s="3">
+      <c r="B101" t="s" s="3">
         <v>33</v>
       </c>
-      <c r="C98" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D98" t="s" s="3">
+      <c r="C101" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D101" t="s" s="3">
         <v>34</v>
       </c>
-      <c r="E98" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F98" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="s" s="1">
+      <c r="E101" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F101" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n" s="4">
+        <v>6.0</v>
+      </c>
+      <c r="B102" t="s" s="3">
         <v>35</v>
       </c>
-      <c r="B99" t="s" s="0">
+      <c r="C102" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D102" t="s" s="3">
         <v>36</v>
+      </c>
+      <c r="E102" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F102" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B103" t="s" s="0">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B106" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C106" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E106" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B107" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="E107" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="B108" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B109" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C109" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D109" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E109" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F109" t="s" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B110" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C110" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D110" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E110" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F110" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="B111" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="C111" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D111" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E111" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F111" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="B112" t="s" s="3">
+        <v>31</v>
+      </c>
+      <c r="C112" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D112" t="s" s="3">
+        <v>32</v>
+      </c>
+      <c r="E112" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F112" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="B113" t="s" s="3">
+        <v>33</v>
+      </c>
+      <c r="C113" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D113" t="s" s="3">
+        <v>34</v>
+      </c>
+      <c r="E113" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F113" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="B114" t="s" s="3">
+        <v>62</v>
+      </c>
+      <c r="C114" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D114" t="s" s="3">
+        <v>32</v>
+      </c>
+      <c r="E114" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F114" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n" s="4">
+        <v>6.0</v>
+      </c>
+      <c r="B115" t="s" s="3">
+        <v>33</v>
+      </c>
+      <c r="C115" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D115" t="s" s="3">
+        <v>34</v>
+      </c>
+      <c r="E115" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F115" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n" s="4">
+        <v>7.0</v>
+      </c>
+      <c r="B116" t="s" s="3">
+        <v>35</v>
+      </c>
+      <c r="C116" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D116" t="s" s="3">
+        <v>36</v>
+      </c>
+      <c r="E116" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F116" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B117" t="s" s="0">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B120" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="C120" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E120" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B121" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E121" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="B122" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B123" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C123" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D123" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E123" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F123" t="s" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B124" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C124" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D124" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E124" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F124" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="B125" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="C125" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D125" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E125" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F125" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="B126" t="s" s="3">
+        <v>31</v>
+      </c>
+      <c r="C126" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D126" t="s" s="3">
+        <v>32</v>
+      </c>
+      <c r="E126" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F126" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="B127" t="s" s="3">
+        <v>56</v>
+      </c>
+      <c r="C127" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D127" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E127" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F127" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="B128" t="s" s="3">
+        <v>31</v>
+      </c>
+      <c r="C128" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D128" t="s" s="3">
+        <v>32</v>
+      </c>
+      <c r="E128" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F128" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n" s="4">
+        <v>6.0</v>
+      </c>
+      <c r="B129" t="s" s="3">
+        <v>33</v>
+      </c>
+      <c r="C129" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D129" t="s" s="3">
+        <v>34</v>
+      </c>
+      <c r="E129" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F129" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n" s="4">
+        <v>7.0</v>
+      </c>
+      <c r="B130" t="s" s="3">
+        <v>35</v>
+      </c>
+      <c r="C130" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D130" t="s" s="3">
+        <v>36</v>
+      </c>
+      <c r="E130" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F130" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B131" t="s" s="0">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B134" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="C134" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E134" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B135" t="s" s="0">
+        <v>66</v>
+      </c>
+      <c r="E135" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="B136" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B137" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C137" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D137" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E137" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F137" t="s" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B138" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C138" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D138" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E138" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F138" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="B139" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="C139" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D139" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E139" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F139" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="B140" t="s" s="3">
+        <v>67</v>
+      </c>
+      <c r="C140" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D140" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E140" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F140" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="B141" t="s" s="3">
+        <v>31</v>
+      </c>
+      <c r="C141" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D141" t="s" s="3">
+        <v>32</v>
+      </c>
+      <c r="E141" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F141" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="B142" t="s" s="3">
+        <v>33</v>
+      </c>
+      <c r="C142" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D142" t="s" s="3">
+        <v>34</v>
+      </c>
+      <c r="E142" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F142" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n" s="4">
+        <v>6.0</v>
+      </c>
+      <c r="B143" t="s" s="3">
+        <v>35</v>
+      </c>
+      <c r="C143" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D143" t="s" s="3">
+        <v>36</v>
+      </c>
+      <c r="E143" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F143" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B144" t="s" s="0">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>